<commit_message>
Exhibits: adopt revised index, dedupe, add Tier-1/2 evidence, team-page capture & preservation letter; merged rebuttal w/ appendix; taxonomy & open-items updates
</commit_message>
<xml_diff>
--- a/99_ARCHIVE/original-tree/EEOC 5.25.27 INVESTIGATION/UPDATED TIMELINE 5.25.26.xlsx
+++ b/99_ARCHIVE/original-tree/EEOC 5.25.27 INVESTIGATION/UPDATED TIMELINE 5.25.26.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10517"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10621"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/langworthylord/Desktop/EEOC 5.21.27 DETAILS/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/langworthylord/GH-Repo/Discrimination-Case/99_ARCHIVE/original-tree/EEOC 5.25.27 INVESTIGATION/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{BE6BE7A2-DE7E-9648-9C7B-7D91321B5565}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1BBBBC4A-C655-6341-8507-3DD1991BD8F4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4080" yWindow="4540" windowWidth="34200" windowHeight="19820" xr2:uid="{AB88D130-70A5-2F4E-9199-408625F92DC5}"/>
+    <workbookView xWindow="5320" yWindow="1140" windowWidth="34200" windowHeight="19600" xr2:uid="{AB88D130-70A5-2F4E-9199-408625F92DC5}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -2406,11 +2406,11 @@
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="25" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -2774,12 +2774,12 @@
       </c>
     </row>
     <row r="2" spans="1:5" ht="48" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="66" t="s">
+      <c r="A2" s="67" t="s">
         <v>327</v>
       </c>
-      <c r="B2" s="66"/>
-      <c r="C2" s="66"/>
-      <c r="D2" s="66"/>
+      <c r="B2" s="67"/>
+      <c r="C2" s="67"/>
+      <c r="D2" s="67"/>
       <c r="E2" s="65"/>
     </row>
     <row r="3" spans="1:5" ht="105" x14ac:dyDescent="0.2">
@@ -2839,7 +2839,7 @@
     </row>
     <row r="7" spans="1:5" ht="45" x14ac:dyDescent="0.2">
       <c r="A7" s="13">
-        <v>46345</v>
+        <v>45615</v>
       </c>
       <c r="B7" s="13" t="s">
         <v>94</v>
@@ -4494,7 +4494,7 @@
       </c>
     </row>
     <row r="120" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A120" s="67" t="s">
+      <c r="A120" s="66" t="s">
         <v>374</v>
       </c>
       <c r="B120" s="31"/>

</xml_diff>